<commit_message>
feat(calculators): implementing 4.7.1.2 method 2 manure methane
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/4.7-other-livestock-manure.xlsx
+++ b/packages/calculators/src/modules/test/4.7-other-livestock-manure.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddiesholl/Code/aginnovationaustralia/emissions-calculators/packages/calculators/src/modules/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47116608-09EC-0345-95F2-F5B53AF80DF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BEE1AAC-71EE-1A42-95E6-0B8A507DDCD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51360" yWindow="6120" windowWidth="28800" windowHeight="25760" xr2:uid="{5678E890-3691-CF46-80E7-00FB1F103661}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="93">
   <si>
     <t>Livestock type</t>
   </si>
@@ -135,15 +135,6 @@
   </si>
   <si>
     <t>MAT</t>
-  </si>
-  <si>
-    <t>≤10</t>
-  </si>
-  <si>
-    <t>≥28</t>
-  </si>
-  <si>
-    <t>Climate zone</t>
   </si>
   <si>
     <t>State</t>
@@ -404,6 +395,18 @@
   </si>
   <si>
     <t>FracGASMSoil</t>
+  </si>
+  <si>
+    <t>Temperature zone</t>
+  </si>
+  <si>
+    <t>input (method 2)</t>
+  </si>
+  <si>
+    <t>10 or below</t>
+  </si>
+  <si>
+    <t>28 or above</t>
   </si>
 </sst>
 </file>
@@ -840,7 +843,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78A5655F-5BFE-554E-A3D3-9DFA9517010F}">
-  <dimension ref="A1:AM55"/>
+  <dimension ref="A1:AM64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="17.33203125" style="3" customWidth="1"/>
@@ -848,7 +851,8 @@
     <col min="3" max="3" width="17.83203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="26.6640625" customWidth="1"/>
     <col min="5" max="5" width="29.6640625" customWidth="1"/>
-    <col min="6" max="7" width="12.1640625" customWidth="1"/>
+    <col min="6" max="6" width="15.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.1640625" customWidth="1"/>
     <col min="8" max="8" width="5.5" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="8.33203125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="13.33203125" bestFit="1" customWidth="1"/>
@@ -886,18 +890,18 @@
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
       <c r="Z3" s="1" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="AA3" s="1"/>
       <c r="AB3" s="1"/>
       <c r="AG3" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="AH3">
         <v>0.21</v>
       </c>
       <c r="AJ3" s="7" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="AK3">
         <v>0.24</v>
@@ -907,6 +911,9 @@
       <c r="C4">
         <v>1776</v>
       </c>
+      <c r="F4">
+        <v>1779</v>
+      </c>
       <c r="I4">
         <v>1783</v>
       </c>
@@ -953,17 +960,17 @@
         <v>1779</v>
       </c>
       <c r="Z4" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="AG4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AH4">
         <f>44/28</f>
         <v>1.5714285714285714</v>
       </c>
       <c r="AJ4" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="AK4">
         <v>0.11</v>
@@ -971,61 +978,64 @@
     </row>
     <row r="5" spans="1:39">
       <c r="C5" t="s">
+        <v>87</v>
+      </c>
+      <c r="F5" t="s">
         <v>90</v>
       </c>
       <c r="I5" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="J5" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="L5" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="M5" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="N5" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="O5" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="P5" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="Q5" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="R5" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="S5" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="T5" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="U5" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="V5" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="W5" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="Y5" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="AG5" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="AH5">
         <v>0.6784</v>
       </c>
       <c r="AJ5" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="AK5">
         <v>0.19</v>
@@ -1035,21 +1045,21 @@
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="AF6" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="AG6" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="AH6">
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="AJ6" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:39">
       <c r="AG7" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="AH7">
         <v>2E-3</v>
@@ -1064,15 +1074,15 @@
     <row r="9" spans="1:39">
       <c r="A9" s="4"/>
       <c r="C9" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="AH9" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="AJ9" s="2"/>
       <c r="AK9" s="2"/>
       <c r="AM9" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:39" ht="17">
@@ -1086,98 +1096,98 @@
         <v>2</v>
       </c>
       <c r="D10" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="F10" t="s">
+        <v>89</v>
+      </c>
+      <c r="G10" t="s">
+        <v>42</v>
+      </c>
+      <c r="H10" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="I10" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="J10" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="L10" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="M10" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="N10" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="O10" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="P10" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q10" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="R10" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="S10" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="E10" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="F10" t="s">
-        <v>35</v>
-      </c>
-      <c r="G10" t="s">
-        <v>45</v>
-      </c>
-      <c r="H10" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="I10" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="J10" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="K10" s="6" t="s">
+      <c r="T10" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="U10" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="V10" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="L10" s="11" t="s">
+      <c r="W10" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="X10" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="Y10" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="Z10" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="M10" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="N10" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="O10" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="P10" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q10" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="R10" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="S10" s="11" t="s">
+      <c r="AA10" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="AB10" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="AC10" s="9" t="s">
         <v>51</v>
-      </c>
-      <c r="T10" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="U10" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="V10" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="W10" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="X10" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="Y10" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="Z10" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="AA10" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="AB10" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="AC10" s="9" t="s">
-        <v>54</v>
       </c>
       <c r="AD10" s="11"/>
       <c r="AE10" s="11"/>
       <c r="AG10" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="AH10" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="AI10" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="AJ10" s="2"/>
       <c r="AK10" s="2"/>
       <c r="AL10" s="2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="AM10" s="2">
         <v>5.8999999999999999E-3</v>
@@ -1194,13 +1204,13 @@
         <v>5</v>
       </c>
       <c r="D11" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E11" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="H11" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="I11">
         <f>VLOOKUP(A11, $AG$11:$AH$18,2,FALSE)</f>
@@ -1211,7 +1221,7 @@
         <v>0.19</v>
       </c>
       <c r="K11" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="L11">
         <f>1-M11</f>
@@ -1289,7 +1299,7 @@
       <c r="AJ11" s="2"/>
       <c r="AK11" s="2"/>
       <c r="AL11" s="2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="AM11" s="2">
         <v>7.0000000000000001E-3</v>
@@ -1306,13 +1316,13 @@
         <v>6</v>
       </c>
       <c r="D12" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E12" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="H12" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="I12">
         <f>VLOOKUP(A12, $AG$11:$AH$18,2,FALSE)</f>
@@ -1323,7 +1333,7 @@
         <v>0.19</v>
       </c>
       <c r="K12" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="L12">
         <f>1-M12</f>
@@ -1401,7 +1411,7 @@
       <c r="AJ12" s="2"/>
       <c r="AK12" s="2"/>
       <c r="AL12" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="AM12" s="2">
         <v>1.8E-3</v>
@@ -1418,13 +1428,13 @@
         <v>7</v>
       </c>
       <c r="D13" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="H13" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="I13">
         <f t="shared" ref="I13:I30" si="0">VLOOKUP(A13, $AG$11:$AH$18,2,FALSE)</f>
@@ -1435,7 +1445,7 @@
         <v>0.19</v>
       </c>
       <c r="K13" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="L13">
         <f t="shared" ref="L13:L30" si="2">1-M13</f>
@@ -1513,7 +1523,7 @@
       <c r="AJ13" s="2"/>
       <c r="AK13" s="2"/>
       <c r="AL13" s="2" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="AM13" s="2">
         <v>2.8999999999999998E-3</v>
@@ -1530,13 +1540,13 @@
         <v>8</v>
       </c>
       <c r="D14" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="H14" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="I14">
         <f t="shared" si="0"/>
@@ -1547,7 +1557,7 @@
         <v>0.19</v>
       </c>
       <c r="K14" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="L14">
         <f t="shared" si="2"/>
@@ -1625,7 +1635,7 @@
       <c r="AJ14" s="2"/>
       <c r="AK14" s="2"/>
       <c r="AL14" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="AM14" s="2">
         <v>8.0000000000000002E-3</v>
@@ -1642,13 +1652,13 @@
         <v>9</v>
       </c>
       <c r="D15" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="H15" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="I15">
         <f t="shared" si="0"/>
@@ -1659,7 +1669,7 @@
         <v>0.19</v>
       </c>
       <c r="K15" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="L15">
         <f t="shared" si="2"/>
@@ -1737,7 +1747,7 @@
       <c r="AJ15" s="2"/>
       <c r="AK15" s="2"/>
       <c r="AL15" s="2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="AM15" s="2">
         <v>1.9900000000000001E-2</v>
@@ -1754,10 +1764,10 @@
         <v>10</v>
       </c>
       <c r="D16" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="H16" s="2" t="s">
         <v>28</v>
@@ -1771,7 +1781,7 @@
         <v>0.19</v>
       </c>
       <c r="K16" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="L16">
         <f t="shared" si="2"/>
@@ -1849,7 +1859,7 @@
       <c r="AJ16" s="2"/>
       <c r="AK16" s="2"/>
       <c r="AL16" s="2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="AM16" s="2">
         <v>5.3E-3</v>
@@ -1866,13 +1876,13 @@
         <v>11</v>
       </c>
       <c r="D17" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="I17">
         <f t="shared" si="0"/>
@@ -1883,7 +1893,7 @@
         <v>0.19</v>
       </c>
       <c r="K17" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="L17">
         <f t="shared" si="2"/>
@@ -1961,7 +1971,7 @@
       <c r="AJ17" s="2"/>
       <c r="AK17" s="2"/>
       <c r="AL17" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="AM17" s="2">
         <v>6.4000000000000003E-3</v>
@@ -1978,13 +1988,13 @@
         <v>12</v>
       </c>
       <c r="D18" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="I18">
         <f t="shared" si="0"/>
@@ -1995,7 +2005,7 @@
         <v>0.19</v>
       </c>
       <c r="K18" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="L18">
         <f t="shared" si="2"/>
@@ -2062,7 +2072,7 @@
         <v>9.0217403904000024E-4</v>
       </c>
       <c r="AG18" s="2" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="AH18" s="2">
         <v>0.34</v>
@@ -2073,7 +2083,7 @@
       <c r="AJ18" s="2"/>
       <c r="AK18" s="10"/>
       <c r="AL18" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="AM18" s="2">
         <v>2.5999999999999999E-3</v>
@@ -2090,13 +2100,13 @@
         <v>13</v>
       </c>
       <c r="D19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="I19">
         <f t="shared" si="0"/>
@@ -2107,7 +2117,7 @@
         <v>0.19</v>
       </c>
       <c r="K19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="L19">
         <f t="shared" si="2"/>
@@ -2176,7 +2186,7 @@
       <c r="AJ19" s="2"/>
       <c r="AK19" s="10"/>
       <c r="AL19" s="2" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="AM19" s="2">
         <v>3.0000000000000001E-3</v>
@@ -2193,13 +2203,13 @@
         <v>14</v>
       </c>
       <c r="D20" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I20">
         <f t="shared" si="0"/>
@@ -2210,7 +2220,7 @@
         <v>0.19</v>
       </c>
       <c r="K20" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="L20">
         <f t="shared" si="2"/>
@@ -2279,7 +2289,7 @@
       <c r="AJ20" s="2"/>
       <c r="AK20" s="2"/>
       <c r="AL20" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="AM20" s="2">
         <v>5.0000000000000001E-3</v>
@@ -2296,13 +2306,13 @@
         <v>15</v>
       </c>
       <c r="D21" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="I21">
         <f t="shared" si="0"/>
@@ -2313,7 +2323,7 @@
         <v>0.19</v>
       </c>
       <c r="K21" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="L21">
         <f t="shared" si="2"/>
@@ -2388,7 +2398,7 @@
       <c r="AJ21" s="2"/>
       <c r="AK21" s="2"/>
       <c r="AL21" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="AM21" s="2">
         <v>2.5999999999999999E-3</v>
@@ -2405,13 +2415,13 @@
         <v>16</v>
       </c>
       <c r="D22" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="I22">
         <f t="shared" si="0"/>
@@ -2422,7 +2432,7 @@
         <v>0.19</v>
       </c>
       <c r="K22" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="L22">
         <f t="shared" si="2"/>
@@ -2492,7 +2502,7 @@
         <v>27</v>
       </c>
       <c r="AL22" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="AM22" s="2">
         <v>1.8E-3</v>
@@ -2509,13 +2519,13 @@
         <v>17</v>
       </c>
       <c r="D23" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="I23">
         <f t="shared" si="0"/>
@@ -2526,7 +2536,7 @@
         <v>0.19</v>
       </c>
       <c r="K23" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="L23">
         <f t="shared" si="2"/>
@@ -2611,10 +2621,10 @@
         <v>18</v>
       </c>
       <c r="D24" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="H24" s="2" t="s">
         <v>28</v>
@@ -2628,7 +2638,7 @@
         <v>0.19</v>
       </c>
       <c r="K24" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="L24">
         <f t="shared" si="2"/>
@@ -2695,7 +2705,7 @@
         <v>3.0798248539968022E-2</v>
       </c>
       <c r="AG24" s="2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="AH24" s="2">
         <v>0.75</v>
@@ -2714,13 +2724,13 @@
         <v>19</v>
       </c>
       <c r="D25" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="I25">
         <f t="shared" si="0"/>
@@ -2731,7 +2741,7 @@
         <v>0.19</v>
       </c>
       <c r="K25" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="L25">
         <f t="shared" si="2"/>
@@ -2798,7 +2808,7 @@
         <v>3.4136148990944033E-2</v>
       </c>
       <c r="AG25" s="2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="AH25" s="2">
         <v>0.8</v>
@@ -2817,13 +2827,13 @@
         <v>20</v>
       </c>
       <c r="D26" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="I26">
         <f t="shared" si="0"/>
@@ -2834,7 +2844,7 @@
         <v>0.19</v>
       </c>
       <c r="K26" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="L26">
         <f t="shared" si="2"/>
@@ -2901,7 +2911,7 @@
         <v>0.11422028619456009</v>
       </c>
       <c r="AG26" s="2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="AH26" s="2">
         <v>0.78</v>
@@ -2920,13 +2930,13 @@
         <v>21</v>
       </c>
       <c r="D27" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="I27">
         <f t="shared" si="0"/>
@@ -2937,7 +2947,7 @@
         <v>0.19</v>
       </c>
       <c r="K27" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="L27">
         <f t="shared" si="2"/>
@@ -3004,7 +3014,7 @@
         <v>1.4600583098304016E-2</v>
       </c>
       <c r="AG27" s="2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="AH27" s="2">
         <v>0.74</v>
@@ -3023,13 +3033,13 @@
         <v>22</v>
       </c>
       <c r="D28" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I28">
         <f t="shared" si="0"/>
@@ -3040,7 +3050,7 @@
         <v>0.19</v>
       </c>
       <c r="K28" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="L28">
         <f t="shared" si="2"/>
@@ -3107,7 +3117,7 @@
         <v>0.11716537914681611</v>
       </c>
       <c r="AG28" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="AH28" s="2">
         <v>0.7</v>
@@ -3126,13 +3136,13 @@
         <v>23</v>
       </c>
       <c r="D29" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="I29">
         <f t="shared" si="0"/>
@@ -3143,7 +3153,7 @@
         <v>0.19</v>
       </c>
       <c r="K29" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="L29">
         <f t="shared" si="2"/>
@@ -3210,7 +3220,7 @@
         <v>3.8860970305248023E-2</v>
       </c>
       <c r="AG29" s="2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="AH29" s="2">
         <v>0.74</v>
@@ -3220,7 +3230,7 @@
     </row>
     <row r="30" spans="1:39">
       <c r="A30" s="2" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>23</v>
@@ -3229,13 +3239,13 @@
         <v>24</v>
       </c>
       <c r="D30" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="I30">
         <f t="shared" si="0"/>
@@ -3246,7 +3256,7 @@
         <v>0.19</v>
       </c>
       <c r="K30" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="L30">
         <f t="shared" si="2"/>
@@ -3313,7 +3323,7 @@
         <v>1.5918572990976015E-2</v>
       </c>
       <c r="AG30" s="2" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="AH30" s="2">
         <v>0.76</v>
@@ -3331,37 +3341,37 @@
         <v>30</v>
       </c>
     </row>
-    <row r="33" spans="5:34">
+    <row r="33" spans="1:34">
       <c r="E33" s="2"/>
       <c r="AG33">
         <v>4.7000000000000002E-3</v>
       </c>
     </row>
-    <row r="34" spans="5:34">
+    <row r="34" spans="1:34">
       <c r="E34" s="2"/>
     </row>
-    <row r="35" spans="5:34">
+    <row r="35" spans="1:34">
       <c r="E35" s="2"/>
       <c r="AG35" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="36" spans="5:34">
+    <row r="36" spans="1:34">
       <c r="E36" s="2"/>
       <c r="AG36" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="37" spans="5:34">
+    <row r="37" spans="1:34">
       <c r="E37" s="2"/>
       <c r="AG37" t="s">
-        <v>33</v>
+        <v>91</v>
       </c>
       <c r="AH37">
         <v>0.66</v>
       </c>
     </row>
-    <row r="38" spans="5:34">
+    <row r="38" spans="1:34">
       <c r="E38" s="2"/>
       <c r="AG38">
         <v>11</v>
@@ -3370,7 +3380,7 @@
         <v>0.68</v>
       </c>
     </row>
-    <row r="39" spans="5:34">
+    <row r="39" spans="1:34">
       <c r="AG39">
         <v>12</v>
       </c>
@@ -3378,7 +3388,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="40" spans="5:34">
+    <row r="40" spans="1:34">
       <c r="AG40">
         <v>13</v>
       </c>
@@ -3386,7 +3396,103 @@
         <v>0.71</v>
       </c>
     </row>
-    <row r="41" spans="5:34">
+    <row r="41" spans="1:34" ht="17">
+      <c r="A41" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C41">
+        <v>5</v>
+      </c>
+      <c r="D41" t="s">
+        <v>56</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F41" t="s">
+        <v>91</v>
+      </c>
+      <c r="H41" t="s">
+        <v>66</v>
+      </c>
+      <c r="I41">
+        <f>VLOOKUP(A41, $AG$11:$AH$18,2,FALSE)</f>
+        <v>2.73</v>
+      </c>
+      <c r="J41">
+        <f>$AK$5</f>
+        <v>0.19</v>
+      </c>
+      <c r="K41" t="s">
+        <v>57</v>
+      </c>
+      <c r="L41">
+        <f>1-M41</f>
+        <v>5.0000000000000044E-2</v>
+      </c>
+      <c r="M41">
+        <f>IF(K41="yes", 1, 0.95)</f>
+        <v>0.95</v>
+      </c>
+      <c r="N41">
+        <f>$AH$4</f>
+        <v>1.5714285714285714</v>
+      </c>
+      <c r="O41">
+        <f>VLOOKUP(A41, $AG$11:$AI$18,3,FALSE)</f>
+        <v>39.5</v>
+      </c>
+      <c r="P41">
+        <f>VLOOKUP(E41,$AL$10:$AM$22,2,FALSE)</f>
+        <v>5.8999999999999999E-3</v>
+      </c>
+      <c r="Q41">
+        <f>IF(D41="yes", 1, 0)</f>
+        <v>1</v>
+      </c>
+      <c r="S41">
+        <f>$AK$3</f>
+        <v>0.24</v>
+      </c>
+      <c r="T41">
+        <f>$AK$4</f>
+        <v>0.11</v>
+      </c>
+      <c r="U41">
+        <f>$AH$5</f>
+        <v>0.6784</v>
+      </c>
+      <c r="W41">
+        <f>VLOOKUP(F41, $AG$37:$AH$55, 2, FALSE)</f>
+        <v>0.66</v>
+      </c>
+      <c r="X41">
+        <f>I41*J41*L41*W41*U41</f>
+        <v>1.1612240640000012E-2</v>
+      </c>
+      <c r="Y41">
+        <f>$AG$33</f>
+        <v>4.7000000000000002E-3</v>
+      </c>
+      <c r="Z41">
+        <f>I41*J41*M41*Y41*U41</f>
+        <v>1.5711713472E-3</v>
+      </c>
+      <c r="AA41">
+        <f>C41*X41*365</f>
+        <v>21.192339168000025</v>
+      </c>
+      <c r="AB41">
+        <f>C41*Z41*365</f>
+        <v>2.8673877086399999</v>
+      </c>
+      <c r="AC41">
+        <f>(AA41+AB41)*10^-3</f>
+        <v>2.4059726876640024E-2</v>
+      </c>
       <c r="AG41">
         <v>14</v>
       </c>
@@ -3394,7 +3500,103 @@
         <v>0.73</v>
       </c>
     </row>
-    <row r="42" spans="5:34">
+    <row r="42" spans="1:34" ht="17">
+      <c r="A42" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C42">
+        <v>6</v>
+      </c>
+      <c r="D42" t="s">
+        <v>57</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F42">
+        <v>11</v>
+      </c>
+      <c r="H42" t="s">
+        <v>66</v>
+      </c>
+      <c r="I42">
+        <f>VLOOKUP(A42, $AG$11:$AH$18,2,FALSE)</f>
+        <v>2.73</v>
+      </c>
+      <c r="J42">
+        <f>$AK$5</f>
+        <v>0.19</v>
+      </c>
+      <c r="K42" t="s">
+        <v>57</v>
+      </c>
+      <c r="L42">
+        <f>1-M42</f>
+        <v>5.0000000000000044E-2</v>
+      </c>
+      <c r="M42">
+        <f>IF(K42="yes", 1, 0.95)</f>
+        <v>0.95</v>
+      </c>
+      <c r="N42">
+        <f>$AH$4</f>
+        <v>1.5714285714285714</v>
+      </c>
+      <c r="O42">
+        <f>VLOOKUP(A42, $AG$11:$AI$18,3,FALSE)</f>
+        <v>39.5</v>
+      </c>
+      <c r="P42">
+        <f>VLOOKUP(E42,$AL$10:$AM$22,2,FALSE)</f>
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="Q42">
+        <f>IF(D42="yes", 1, 0)</f>
+        <v>0</v>
+      </c>
+      <c r="S42">
+        <f>$AK$3</f>
+        <v>0.24</v>
+      </c>
+      <c r="T42">
+        <f>$AK$4</f>
+        <v>0.11</v>
+      </c>
+      <c r="U42">
+        <f>$AH$5</f>
+        <v>0.6784</v>
+      </c>
+      <c r="W42">
+        <f t="shared" ref="W42:W60" si="18">VLOOKUP(F42, $AG$37:$AH$55, 2, FALSE)</f>
+        <v>0.68</v>
+      </c>
+      <c r="X42">
+        <f>I42*J42*L42*W42*U42</f>
+        <v>1.1964126720000011E-2</v>
+      </c>
+      <c r="Y42">
+        <f>$AG$33</f>
+        <v>4.7000000000000002E-3</v>
+      </c>
+      <c r="Z42">
+        <f>I42*J42*M42*Y42*U42</f>
+        <v>1.5711713472E-3</v>
+      </c>
+      <c r="AA42">
+        <f>C42*X42*365</f>
+        <v>26.201437516800027</v>
+      </c>
+      <c r="AB42">
+        <f>C42*Z42*365</f>
+        <v>3.4408652503679997</v>
+      </c>
+      <c r="AC42">
+        <f>(AA42+AB42)*10^-3</f>
+        <v>2.9642302767168026E-2</v>
+      </c>
       <c r="AG42">
         <v>15</v>
       </c>
@@ -3402,7 +3604,103 @@
         <v>0.74</v>
       </c>
     </row>
-    <row r="43" spans="5:34">
+    <row r="43" spans="1:34" ht="17">
+      <c r="A43" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C43">
+        <v>7</v>
+      </c>
+      <c r="D43" t="s">
+        <v>56</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F43">
+        <v>12</v>
+      </c>
+      <c r="H43" t="s">
+        <v>66</v>
+      </c>
+      <c r="I43">
+        <f t="shared" ref="I43:I60" si="19">VLOOKUP(A43, $AG$11:$AH$18,2,FALSE)</f>
+        <v>2.73</v>
+      </c>
+      <c r="J43">
+        <f t="shared" ref="J43:J60" si="20">$AK$5</f>
+        <v>0.19</v>
+      </c>
+      <c r="K43" t="s">
+        <v>57</v>
+      </c>
+      <c r="L43">
+        <f t="shared" ref="L43:L60" si="21">1-M43</f>
+        <v>5.0000000000000044E-2</v>
+      </c>
+      <c r="M43">
+        <f t="shared" ref="M43:M60" si="22">IF(K43="yes", 1, 0.95)</f>
+        <v>0.95</v>
+      </c>
+      <c r="N43">
+        <f t="shared" ref="N43:N60" si="23">$AH$4</f>
+        <v>1.5714285714285714</v>
+      </c>
+      <c r="O43">
+        <f t="shared" ref="O43:O60" si="24">VLOOKUP(A43, $AG$11:$AI$18,3,FALSE)</f>
+        <v>39.5</v>
+      </c>
+      <c r="P43">
+        <f t="shared" ref="P43:P60" si="25">VLOOKUP(E43,$AL$10:$AM$22,2,FALSE)</f>
+        <v>1.8E-3</v>
+      </c>
+      <c r="Q43">
+        <f t="shared" ref="Q43:Q60" si="26">IF(D43="yes", 1, 0)</f>
+        <v>1</v>
+      </c>
+      <c r="S43">
+        <f t="shared" ref="S43:S60" si="27">$AK$3</f>
+        <v>0.24</v>
+      </c>
+      <c r="T43">
+        <f t="shared" ref="T43:T60" si="28">$AK$4</f>
+        <v>0.11</v>
+      </c>
+      <c r="U43">
+        <f t="shared" ref="U43:U60" si="29">$AH$5</f>
+        <v>0.6784</v>
+      </c>
+      <c r="W43">
+        <f t="shared" si="18"/>
+        <v>0.7</v>
+      </c>
+      <c r="X43">
+        <f t="shared" ref="X43:X60" si="30">I43*J43*L43*W43*U43</f>
+        <v>1.231601280000001E-2</v>
+      </c>
+      <c r="Y43">
+        <f t="shared" ref="Y43:Y60" si="31">$AG$33</f>
+        <v>4.7000000000000002E-3</v>
+      </c>
+      <c r="Z43">
+        <f t="shared" ref="Z43:Z60" si="32">I43*J43*M43*Y43*U43</f>
+        <v>1.5711713472E-3</v>
+      </c>
+      <c r="AA43">
+        <f t="shared" ref="AA43:AA60" si="33">C43*X43*365</f>
+        <v>31.467412704000026</v>
+      </c>
+      <c r="AB43">
+        <f t="shared" ref="AB43:AB60" si="34">C43*Z43*365</f>
+        <v>4.0143427920960004</v>
+      </c>
+      <c r="AC43">
+        <f t="shared" ref="AC43:AC60" si="35">(AA43+AB43)*10^-3</f>
+        <v>3.5481755496096029E-2</v>
+      </c>
       <c r="AG43">
         <v>16</v>
       </c>
@@ -3410,7 +3708,103 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="44" spans="5:34">
+    <row r="44" spans="1:34" ht="17">
+      <c r="A44" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C44">
+        <v>8</v>
+      </c>
+      <c r="D44" t="s">
+        <v>57</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F44">
+        <v>13</v>
+      </c>
+      <c r="H44" t="s">
+        <v>66</v>
+      </c>
+      <c r="I44">
+        <f t="shared" si="19"/>
+        <v>2.73</v>
+      </c>
+      <c r="J44">
+        <f t="shared" si="20"/>
+        <v>0.19</v>
+      </c>
+      <c r="K44" t="s">
+        <v>57</v>
+      </c>
+      <c r="L44">
+        <f t="shared" si="21"/>
+        <v>5.0000000000000044E-2</v>
+      </c>
+      <c r="M44">
+        <f t="shared" si="22"/>
+        <v>0.95</v>
+      </c>
+      <c r="N44">
+        <f t="shared" si="23"/>
+        <v>1.5714285714285714</v>
+      </c>
+      <c r="O44">
+        <f t="shared" si="24"/>
+        <v>39.5</v>
+      </c>
+      <c r="P44">
+        <f t="shared" si="25"/>
+        <v>2.8999999999999998E-3</v>
+      </c>
+      <c r="Q44">
+        <f t="shared" si="26"/>
+        <v>0</v>
+      </c>
+      <c r="S44">
+        <f t="shared" si="27"/>
+        <v>0.24</v>
+      </c>
+      <c r="T44">
+        <f t="shared" si="28"/>
+        <v>0.11</v>
+      </c>
+      <c r="U44">
+        <f t="shared" si="29"/>
+        <v>0.6784</v>
+      </c>
+      <c r="W44">
+        <f t="shared" si="18"/>
+        <v>0.71</v>
+      </c>
+      <c r="X44">
+        <f t="shared" si="30"/>
+        <v>1.2491955840000011E-2</v>
+      </c>
+      <c r="Y44">
+        <f t="shared" si="31"/>
+        <v>4.7000000000000002E-3</v>
+      </c>
+      <c r="Z44">
+        <f t="shared" si="32"/>
+        <v>1.5711713472E-3</v>
+      </c>
+      <c r="AA44">
+        <f t="shared" si="33"/>
+        <v>36.476511052800035</v>
+      </c>
+      <c r="AB44">
+        <f t="shared" si="34"/>
+        <v>4.5878203338240002</v>
+      </c>
+      <c r="AC44">
+        <f t="shared" si="35"/>
+        <v>4.1064331386624034E-2</v>
+      </c>
       <c r="AG44">
         <v>17</v>
       </c>
@@ -3418,7 +3812,103 @@
         <v>0.76</v>
       </c>
     </row>
-    <row r="45" spans="5:34">
+    <row r="45" spans="1:34" ht="17">
+      <c r="A45" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C45">
+        <v>9</v>
+      </c>
+      <c r="D45" t="s">
+        <v>56</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F45">
+        <v>14</v>
+      </c>
+      <c r="H45" t="s">
+        <v>66</v>
+      </c>
+      <c r="I45">
+        <f t="shared" si="19"/>
+        <v>0.34</v>
+      </c>
+      <c r="J45">
+        <f t="shared" si="20"/>
+        <v>0.19</v>
+      </c>
+      <c r="K45" t="s">
+        <v>57</v>
+      </c>
+      <c r="L45">
+        <f t="shared" si="21"/>
+        <v>5.0000000000000044E-2</v>
+      </c>
+      <c r="M45">
+        <f t="shared" si="22"/>
+        <v>0.95</v>
+      </c>
+      <c r="N45">
+        <f t="shared" si="23"/>
+        <v>1.5714285714285714</v>
+      </c>
+      <c r="O45">
+        <f t="shared" si="24"/>
+        <v>7</v>
+      </c>
+      <c r="P45">
+        <f t="shared" si="25"/>
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="Q45">
+        <f t="shared" si="26"/>
+        <v>1</v>
+      </c>
+      <c r="S45">
+        <f t="shared" si="27"/>
+        <v>0.24</v>
+      </c>
+      <c r="T45">
+        <f t="shared" si="28"/>
+        <v>0.11</v>
+      </c>
+      <c r="U45">
+        <f t="shared" si="29"/>
+        <v>0.6784</v>
+      </c>
+      <c r="W45">
+        <f t="shared" si="18"/>
+        <v>0.73</v>
+      </c>
+      <c r="X45">
+        <f t="shared" si="30"/>
+        <v>1.5995993600000015E-3</v>
+      </c>
+      <c r="Y45">
+        <f t="shared" si="31"/>
+        <v>4.7000000000000002E-3</v>
+      </c>
+      <c r="Z45">
+        <f t="shared" si="32"/>
+        <v>1.9567701760000002E-4</v>
+      </c>
+      <c r="AA45">
+        <f t="shared" si="33"/>
+        <v>5.254683897600005</v>
+      </c>
+      <c r="AB45">
+        <f t="shared" si="34"/>
+        <v>0.64279900281600011</v>
+      </c>
+      <c r="AC45">
+        <f t="shared" si="35"/>
+        <v>5.8974829004160047E-3</v>
+      </c>
       <c r="AG45">
         <v>18</v>
       </c>
@@ -3426,7 +3916,103 @@
         <v>0.77</v>
       </c>
     </row>
-    <row r="46" spans="5:34">
+    <row r="46" spans="1:34" ht="17">
+      <c r="A46" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C46">
+        <v>10</v>
+      </c>
+      <c r="D46" t="s">
+        <v>57</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F46">
+        <v>15</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I46">
+        <f t="shared" si="19"/>
+        <v>0.34</v>
+      </c>
+      <c r="J46">
+        <f t="shared" si="20"/>
+        <v>0.19</v>
+      </c>
+      <c r="K46" t="s">
+        <v>57</v>
+      </c>
+      <c r="L46">
+        <f t="shared" si="21"/>
+        <v>5.0000000000000044E-2</v>
+      </c>
+      <c r="M46">
+        <f t="shared" si="22"/>
+        <v>0.95</v>
+      </c>
+      <c r="N46">
+        <f t="shared" si="23"/>
+        <v>1.5714285714285714</v>
+      </c>
+      <c r="O46">
+        <f t="shared" si="24"/>
+        <v>7</v>
+      </c>
+      <c r="P46">
+        <f t="shared" si="25"/>
+        <v>1.9900000000000001E-2</v>
+      </c>
+      <c r="Q46">
+        <f t="shared" si="26"/>
+        <v>0</v>
+      </c>
+      <c r="S46">
+        <f t="shared" si="27"/>
+        <v>0.24</v>
+      </c>
+      <c r="T46">
+        <f t="shared" si="28"/>
+        <v>0.11</v>
+      </c>
+      <c r="U46">
+        <f t="shared" si="29"/>
+        <v>0.6784</v>
+      </c>
+      <c r="W46">
+        <f t="shared" si="18"/>
+        <v>0.74</v>
+      </c>
+      <c r="X46">
+        <f t="shared" si="30"/>
+        <v>1.6215116800000018E-3</v>
+      </c>
+      <c r="Y46">
+        <f t="shared" si="31"/>
+        <v>4.7000000000000002E-3</v>
+      </c>
+      <c r="Z46">
+        <f t="shared" si="32"/>
+        <v>1.9567701760000002E-4</v>
+      </c>
+      <c r="AA46">
+        <f t="shared" si="33"/>
+        <v>5.9185176320000075</v>
+      </c>
+      <c r="AB46">
+        <f t="shared" si="34"/>
+        <v>0.71422111424000012</v>
+      </c>
+      <c r="AC46">
+        <f t="shared" si="35"/>
+        <v>6.6327387462400073E-3</v>
+      </c>
       <c r="AG46">
         <v>19</v>
       </c>
@@ -3434,7 +4020,103 @@
         <v>0.77</v>
       </c>
     </row>
-    <row r="47" spans="5:34">
+    <row r="47" spans="1:34" ht="17">
+      <c r="A47" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C47">
+        <v>11</v>
+      </c>
+      <c r="D47" t="s">
+        <v>56</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F47">
+        <v>16</v>
+      </c>
+      <c r="H47" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="I47">
+        <f t="shared" si="19"/>
+        <v>0.34</v>
+      </c>
+      <c r="J47">
+        <f t="shared" si="20"/>
+        <v>0.19</v>
+      </c>
+      <c r="K47" t="s">
+        <v>57</v>
+      </c>
+      <c r="L47">
+        <f t="shared" si="21"/>
+        <v>5.0000000000000044E-2</v>
+      </c>
+      <c r="M47">
+        <f t="shared" si="22"/>
+        <v>0.95</v>
+      </c>
+      <c r="N47">
+        <f t="shared" si="23"/>
+        <v>1.5714285714285714</v>
+      </c>
+      <c r="O47">
+        <f t="shared" si="24"/>
+        <v>7</v>
+      </c>
+      <c r="P47">
+        <f t="shared" si="25"/>
+        <v>5.3E-3</v>
+      </c>
+      <c r="Q47">
+        <f t="shared" si="26"/>
+        <v>1</v>
+      </c>
+      <c r="S47">
+        <f t="shared" si="27"/>
+        <v>0.24</v>
+      </c>
+      <c r="T47">
+        <f t="shared" si="28"/>
+        <v>0.11</v>
+      </c>
+      <c r="U47">
+        <f t="shared" si="29"/>
+        <v>0.6784</v>
+      </c>
+      <c r="W47">
+        <f t="shared" si="18"/>
+        <v>0.75</v>
+      </c>
+      <c r="X47">
+        <f t="shared" si="30"/>
+        <v>1.6434240000000016E-3</v>
+      </c>
+      <c r="Y47">
+        <f t="shared" si="31"/>
+        <v>4.7000000000000002E-3</v>
+      </c>
+      <c r="Z47">
+        <f t="shared" si="32"/>
+        <v>1.9567701760000002E-4</v>
+      </c>
+      <c r="AA47">
+        <f t="shared" si="33"/>
+        <v>6.5983473600000062</v>
+      </c>
+      <c r="AB47">
+        <f t="shared" si="34"/>
+        <v>0.78564322566400013</v>
+      </c>
+      <c r="AC47">
+        <f t="shared" si="35"/>
+        <v>7.383990585664006E-3</v>
+      </c>
       <c r="AG47">
         <v>20</v>
       </c>
@@ -3442,7 +4124,103 @@
         <v>0.78</v>
       </c>
     </row>
-    <row r="48" spans="5:34">
+    <row r="48" spans="1:34" ht="17">
+      <c r="A48" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C48">
+        <v>12</v>
+      </c>
+      <c r="D48" t="s">
+        <v>57</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="F48">
+        <v>17</v>
+      </c>
+      <c r="H48" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="I48">
+        <f t="shared" si="19"/>
+        <v>0.34</v>
+      </c>
+      <c r="J48">
+        <f t="shared" si="20"/>
+        <v>0.19</v>
+      </c>
+      <c r="K48" t="s">
+        <v>57</v>
+      </c>
+      <c r="L48">
+        <f t="shared" si="21"/>
+        <v>5.0000000000000044E-2</v>
+      </c>
+      <c r="M48">
+        <f t="shared" si="22"/>
+        <v>0.95</v>
+      </c>
+      <c r="N48">
+        <f t="shared" si="23"/>
+        <v>1.5714285714285714</v>
+      </c>
+      <c r="O48">
+        <f t="shared" si="24"/>
+        <v>7</v>
+      </c>
+      <c r="P48">
+        <f t="shared" si="25"/>
+        <v>6.4000000000000003E-3</v>
+      </c>
+      <c r="Q48">
+        <f t="shared" si="26"/>
+        <v>0</v>
+      </c>
+      <c r="S48">
+        <f t="shared" si="27"/>
+        <v>0.24</v>
+      </c>
+      <c r="T48">
+        <f t="shared" si="28"/>
+        <v>0.11</v>
+      </c>
+      <c r="U48">
+        <f t="shared" si="29"/>
+        <v>0.6784</v>
+      </c>
+      <c r="W48">
+        <f t="shared" si="18"/>
+        <v>0.76</v>
+      </c>
+      <c r="X48">
+        <f t="shared" si="30"/>
+        <v>1.6653363200000019E-3</v>
+      </c>
+      <c r="Y48">
+        <f t="shared" si="31"/>
+        <v>4.7000000000000002E-3</v>
+      </c>
+      <c r="Z48">
+        <f t="shared" si="32"/>
+        <v>1.9567701760000002E-4</v>
+      </c>
+      <c r="AA48">
+        <f t="shared" si="33"/>
+        <v>7.2941730816000083</v>
+      </c>
+      <c r="AB48">
+        <f t="shared" si="34"/>
+        <v>0.85706533708800003</v>
+      </c>
+      <c r="AC48">
+        <f t="shared" si="35"/>
+        <v>8.1512384186880078E-3</v>
+      </c>
       <c r="AG48">
         <v>21</v>
       </c>
@@ -3450,7 +4228,103 @@
         <v>0.78</v>
       </c>
     </row>
-    <row r="49" spans="33:34">
+    <row r="49" spans="1:34" ht="17">
+      <c r="A49" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C49">
+        <v>13</v>
+      </c>
+      <c r="D49" t="s">
+        <v>56</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="F49">
+        <v>18</v>
+      </c>
+      <c r="H49" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="I49">
+        <f t="shared" si="19"/>
+        <v>0.34</v>
+      </c>
+      <c r="J49">
+        <f t="shared" si="20"/>
+        <v>0.19</v>
+      </c>
+      <c r="K49" t="s">
+        <v>57</v>
+      </c>
+      <c r="L49">
+        <f t="shared" si="21"/>
+        <v>5.0000000000000044E-2</v>
+      </c>
+      <c r="M49">
+        <f t="shared" si="22"/>
+        <v>0.95</v>
+      </c>
+      <c r="N49">
+        <f t="shared" si="23"/>
+        <v>1.5714285714285714</v>
+      </c>
+      <c r="O49">
+        <f t="shared" si="24"/>
+        <v>7</v>
+      </c>
+      <c r="P49">
+        <f t="shared" si="25"/>
+        <v>2.5999999999999999E-3</v>
+      </c>
+      <c r="Q49">
+        <f t="shared" si="26"/>
+        <v>1</v>
+      </c>
+      <c r="S49">
+        <f t="shared" si="27"/>
+        <v>0.24</v>
+      </c>
+      <c r="T49">
+        <f t="shared" si="28"/>
+        <v>0.11</v>
+      </c>
+      <c r="U49">
+        <f t="shared" si="29"/>
+        <v>0.6784</v>
+      </c>
+      <c r="W49">
+        <f t="shared" si="18"/>
+        <v>0.77</v>
+      </c>
+      <c r="X49">
+        <f t="shared" si="30"/>
+        <v>1.6872486400000017E-3</v>
+      </c>
+      <c r="Y49">
+        <f t="shared" si="31"/>
+        <v>4.7000000000000002E-3</v>
+      </c>
+      <c r="Z49">
+        <f t="shared" si="32"/>
+        <v>1.9567701760000002E-4</v>
+      </c>
+      <c r="AA49">
+        <f t="shared" si="33"/>
+        <v>8.0059947968000085</v>
+      </c>
+      <c r="AB49">
+        <f t="shared" si="34"/>
+        <v>0.92848744851200005</v>
+      </c>
+      <c r="AC49">
+        <f t="shared" si="35"/>
+        <v>8.9344822453120091E-3</v>
+      </c>
       <c r="AG49">
         <v>22</v>
       </c>
@@ -3458,7 +4332,103 @@
         <v>0.78</v>
       </c>
     </row>
-    <row r="50" spans="33:34">
+    <row r="50" spans="1:34" ht="17">
+      <c r="A50" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C50">
+        <v>14</v>
+      </c>
+      <c r="D50" t="s">
+        <v>57</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="F50">
+        <v>19</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="I50">
+        <f t="shared" si="19"/>
+        <v>0.34</v>
+      </c>
+      <c r="J50">
+        <f t="shared" si="20"/>
+        <v>0.19</v>
+      </c>
+      <c r="K50" t="s">
+        <v>57</v>
+      </c>
+      <c r="L50">
+        <f t="shared" si="21"/>
+        <v>5.0000000000000044E-2</v>
+      </c>
+      <c r="M50">
+        <f t="shared" si="22"/>
+        <v>0.95</v>
+      </c>
+      <c r="N50">
+        <f t="shared" si="23"/>
+        <v>1.5714285714285714</v>
+      </c>
+      <c r="O50">
+        <f t="shared" si="24"/>
+        <v>7</v>
+      </c>
+      <c r="P50">
+        <f t="shared" si="25"/>
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="Q50">
+        <f t="shared" si="26"/>
+        <v>0</v>
+      </c>
+      <c r="S50">
+        <f t="shared" si="27"/>
+        <v>0.24</v>
+      </c>
+      <c r="T50">
+        <f t="shared" si="28"/>
+        <v>0.11</v>
+      </c>
+      <c r="U50">
+        <f t="shared" si="29"/>
+        <v>0.6784</v>
+      </c>
+      <c r="W50">
+        <f t="shared" si="18"/>
+        <v>0.77</v>
+      </c>
+      <c r="X50">
+        <f t="shared" si="30"/>
+        <v>1.6872486400000017E-3</v>
+      </c>
+      <c r="Y50">
+        <f t="shared" si="31"/>
+        <v>4.7000000000000002E-3</v>
+      </c>
+      <c r="Z50">
+        <f t="shared" si="32"/>
+        <v>1.9567701760000002E-4</v>
+      </c>
+      <c r="AA50">
+        <f t="shared" si="33"/>
+        <v>8.6218405504000089</v>
+      </c>
+      <c r="AB50">
+        <f t="shared" si="34"/>
+        <v>0.99990955993600006</v>
+      </c>
+      <c r="AC50">
+        <f t="shared" si="35"/>
+        <v>9.6217501103360095E-3</v>
+      </c>
       <c r="AG50">
         <v>23</v>
       </c>
@@ -3466,7 +4436,103 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="51" spans="33:34">
+    <row r="51" spans="1:34" ht="17">
+      <c r="A51" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C51">
+        <v>15</v>
+      </c>
+      <c r="D51" t="s">
+        <v>56</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F51">
+        <v>20</v>
+      </c>
+      <c r="H51" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="I51">
+        <f t="shared" si="19"/>
+        <v>0.34</v>
+      </c>
+      <c r="J51">
+        <f t="shared" si="20"/>
+        <v>0.19</v>
+      </c>
+      <c r="K51" t="s">
+        <v>56</v>
+      </c>
+      <c r="L51">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="M51">
+        <f t="shared" si="22"/>
+        <v>1</v>
+      </c>
+      <c r="N51">
+        <f t="shared" si="23"/>
+        <v>1.5714285714285714</v>
+      </c>
+      <c r="O51">
+        <f t="shared" si="24"/>
+        <v>7</v>
+      </c>
+      <c r="P51">
+        <f t="shared" si="25"/>
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="Q51">
+        <f t="shared" si="26"/>
+        <v>1</v>
+      </c>
+      <c r="S51">
+        <f t="shared" si="27"/>
+        <v>0.24</v>
+      </c>
+      <c r="T51">
+        <f t="shared" si="28"/>
+        <v>0.11</v>
+      </c>
+      <c r="U51">
+        <f t="shared" si="29"/>
+        <v>0.6784</v>
+      </c>
+      <c r="W51">
+        <f t="shared" si="18"/>
+        <v>0.78</v>
+      </c>
+      <c r="X51">
+        <f t="shared" si="30"/>
+        <v>0</v>
+      </c>
+      <c r="Y51">
+        <f t="shared" si="31"/>
+        <v>4.7000000000000002E-3</v>
+      </c>
+      <c r="Z51">
+        <f t="shared" si="32"/>
+        <v>2.0597580800000003E-4</v>
+      </c>
+      <c r="AA51">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="AB51">
+        <f t="shared" si="34"/>
+        <v>1.1277175488000002</v>
+      </c>
+      <c r="AC51">
+        <f t="shared" si="35"/>
+        <v>1.1277175488000003E-3</v>
+      </c>
       <c r="AG51">
         <v>24</v>
       </c>
@@ -3474,7 +4540,103 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="52" spans="33:34">
+    <row r="52" spans="1:34" ht="17">
+      <c r="A52" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C52">
+        <v>16</v>
+      </c>
+      <c r="D52" t="s">
+        <v>57</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="F52">
+        <v>21</v>
+      </c>
+      <c r="H52" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="I52">
+        <f t="shared" si="19"/>
+        <v>0.91</v>
+      </c>
+      <c r="J52">
+        <f t="shared" si="20"/>
+        <v>0.19</v>
+      </c>
+      <c r="K52" t="s">
+        <v>56</v>
+      </c>
+      <c r="L52">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="M52">
+        <f t="shared" si="22"/>
+        <v>1</v>
+      </c>
+      <c r="N52">
+        <f t="shared" si="23"/>
+        <v>1.5714285714285714</v>
+      </c>
+      <c r="O52">
+        <f t="shared" si="24"/>
+        <v>13.2</v>
+      </c>
+      <c r="P52">
+        <f t="shared" si="25"/>
+        <v>2.5999999999999999E-3</v>
+      </c>
+      <c r="Q52">
+        <f t="shared" si="26"/>
+        <v>0</v>
+      </c>
+      <c r="S52">
+        <f t="shared" si="27"/>
+        <v>0.24</v>
+      </c>
+      <c r="T52">
+        <f t="shared" si="28"/>
+        <v>0.11</v>
+      </c>
+      <c r="U52">
+        <f t="shared" si="29"/>
+        <v>0.6784</v>
+      </c>
+      <c r="W52">
+        <f t="shared" si="18"/>
+        <v>0.78</v>
+      </c>
+      <c r="X52">
+        <f t="shared" si="30"/>
+        <v>0</v>
+      </c>
+      <c r="Y52">
+        <f t="shared" si="31"/>
+        <v>4.7000000000000002E-3</v>
+      </c>
+      <c r="Z52">
+        <f t="shared" si="32"/>
+        <v>5.5128819200000003E-4</v>
+      </c>
+      <c r="AA52">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="AB52">
+        <f t="shared" si="34"/>
+        <v>3.21952304128</v>
+      </c>
+      <c r="AC52">
+        <f t="shared" si="35"/>
+        <v>3.21952304128E-3</v>
+      </c>
       <c r="AG52">
         <v>25</v>
       </c>
@@ -3482,7 +4644,103 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="53" spans="33:34">
+    <row r="53" spans="1:34" ht="17">
+      <c r="A53" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C53">
+        <v>17</v>
+      </c>
+      <c r="D53" t="s">
+        <v>56</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="F53">
+        <v>22</v>
+      </c>
+      <c r="H53" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="I53">
+        <f t="shared" si="19"/>
+        <v>0.91</v>
+      </c>
+      <c r="J53">
+        <f t="shared" si="20"/>
+        <v>0.19</v>
+      </c>
+      <c r="K53" t="s">
+        <v>56</v>
+      </c>
+      <c r="L53">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="M53">
+        <f t="shared" si="22"/>
+        <v>1</v>
+      </c>
+      <c r="N53">
+        <f t="shared" si="23"/>
+        <v>1.5714285714285714</v>
+      </c>
+      <c r="O53">
+        <f t="shared" si="24"/>
+        <v>13.2</v>
+      </c>
+      <c r="P53">
+        <f t="shared" si="25"/>
+        <v>1.8E-3</v>
+      </c>
+      <c r="Q53">
+        <f t="shared" si="26"/>
+        <v>1</v>
+      </c>
+      <c r="S53">
+        <f t="shared" si="27"/>
+        <v>0.24</v>
+      </c>
+      <c r="T53">
+        <f t="shared" si="28"/>
+        <v>0.11</v>
+      </c>
+      <c r="U53">
+        <f t="shared" si="29"/>
+        <v>0.6784</v>
+      </c>
+      <c r="W53">
+        <f t="shared" si="18"/>
+        <v>0.78</v>
+      </c>
+      <c r="X53">
+        <f t="shared" si="30"/>
+        <v>0</v>
+      </c>
+      <c r="Y53">
+        <f t="shared" si="31"/>
+        <v>4.7000000000000002E-3</v>
+      </c>
+      <c r="Z53">
+        <f t="shared" si="32"/>
+        <v>5.5128819200000003E-4</v>
+      </c>
+      <c r="AA53">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="AB53">
+        <f t="shared" si="34"/>
+        <v>3.4207432313599999</v>
+      </c>
+      <c r="AC53">
+        <f t="shared" si="35"/>
+        <v>3.4207432313600001E-3</v>
+      </c>
       <c r="AG53">
         <v>26</v>
       </c>
@@ -3490,7 +4748,103 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="54" spans="33:34">
+    <row r="54" spans="1:34" ht="17">
+      <c r="A54" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C54">
+        <v>18</v>
+      </c>
+      <c r="D54" t="s">
+        <v>57</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F54">
+        <v>23</v>
+      </c>
+      <c r="H54" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I54">
+        <f t="shared" si="19"/>
+        <v>0.91</v>
+      </c>
+      <c r="J54">
+        <f t="shared" si="20"/>
+        <v>0.19</v>
+      </c>
+      <c r="K54" t="s">
+        <v>56</v>
+      </c>
+      <c r="L54">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="M54">
+        <f t="shared" si="22"/>
+        <v>1</v>
+      </c>
+      <c r="N54">
+        <f t="shared" si="23"/>
+        <v>1.5714285714285714</v>
+      </c>
+      <c r="O54">
+        <f t="shared" si="24"/>
+        <v>13.2</v>
+      </c>
+      <c r="P54">
+        <f t="shared" si="25"/>
+        <v>1.8E-3</v>
+      </c>
+      <c r="Q54">
+        <f t="shared" si="26"/>
+        <v>0</v>
+      </c>
+      <c r="S54">
+        <f t="shared" si="27"/>
+        <v>0.24</v>
+      </c>
+      <c r="T54">
+        <f t="shared" si="28"/>
+        <v>0.11</v>
+      </c>
+      <c r="U54">
+        <f t="shared" si="29"/>
+        <v>0.6784</v>
+      </c>
+      <c r="W54">
+        <f t="shared" si="18"/>
+        <v>0.79</v>
+      </c>
+      <c r="X54">
+        <f t="shared" si="30"/>
+        <v>0</v>
+      </c>
+      <c r="Y54">
+        <f t="shared" si="31"/>
+        <v>4.7000000000000002E-3</v>
+      </c>
+      <c r="Z54">
+        <f t="shared" si="32"/>
+        <v>5.5128819200000003E-4</v>
+      </c>
+      <c r="AA54">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="AB54">
+        <f t="shared" si="34"/>
+        <v>3.6219634214399998</v>
+      </c>
+      <c r="AC54">
+        <f t="shared" si="35"/>
+        <v>3.6219634214399998E-3</v>
+      </c>
       <c r="AG54">
         <v>27</v>
       </c>
@@ -3498,13 +4852,611 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="55" spans="33:34">
+    <row r="55" spans="1:34" ht="17">
+      <c r="A55" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C55">
+        <v>19</v>
+      </c>
+      <c r="D55" t="s">
+        <v>56</v>
+      </c>
+      <c r="E55" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F55">
+        <v>24</v>
+      </c>
+      <c r="H55" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="I55">
+        <f t="shared" si="19"/>
+        <v>0.91</v>
+      </c>
+      <c r="J55">
+        <f t="shared" si="20"/>
+        <v>0.19</v>
+      </c>
+      <c r="K55" t="s">
+        <v>56</v>
+      </c>
+      <c r="L55">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="M55">
+        <f t="shared" si="22"/>
+        <v>1</v>
+      </c>
+      <c r="N55">
+        <f t="shared" si="23"/>
+        <v>1.5714285714285714</v>
+      </c>
+      <c r="O55">
+        <f t="shared" si="24"/>
+        <v>13.2</v>
+      </c>
+      <c r="P55">
+        <f t="shared" si="25"/>
+        <v>2.8999999999999998E-3</v>
+      </c>
+      <c r="Q55">
+        <f t="shared" si="26"/>
+        <v>1</v>
+      </c>
+      <c r="S55">
+        <f t="shared" si="27"/>
+        <v>0.24</v>
+      </c>
+      <c r="T55">
+        <f t="shared" si="28"/>
+        <v>0.11</v>
+      </c>
+      <c r="U55">
+        <f t="shared" si="29"/>
+        <v>0.6784</v>
+      </c>
+      <c r="W55">
+        <f t="shared" si="18"/>
+        <v>0.79</v>
+      </c>
+      <c r="X55">
+        <f t="shared" si="30"/>
+        <v>0</v>
+      </c>
+      <c r="Y55">
+        <f t="shared" si="31"/>
+        <v>4.7000000000000002E-3</v>
+      </c>
+      <c r="Z55">
+        <f t="shared" si="32"/>
+        <v>5.5128819200000003E-4</v>
+      </c>
+      <c r="AA55">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="AB55">
+        <f t="shared" si="34"/>
+        <v>3.8231836115200006</v>
+      </c>
+      <c r="AC55">
+        <f t="shared" si="35"/>
+        <v>3.8231836115200008E-3</v>
+      </c>
       <c r="AG55" t="s">
-        <v>34</v>
+        <v>92</v>
       </c>
       <c r="AH55">
         <v>0.8</v>
       </c>
+    </row>
+    <row r="56" spans="1:34">
+      <c r="A56" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C56">
+        <v>20</v>
+      </c>
+      <c r="D56" t="s">
+        <v>57</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F56">
+        <v>25</v>
+      </c>
+      <c r="H56" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="I56">
+        <f t="shared" si="19"/>
+        <v>2.73</v>
+      </c>
+      <c r="J56">
+        <f t="shared" si="20"/>
+        <v>0.19</v>
+      </c>
+      <c r="K56" t="s">
+        <v>56</v>
+      </c>
+      <c r="L56">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="M56">
+        <f t="shared" si="22"/>
+        <v>1</v>
+      </c>
+      <c r="N56">
+        <f t="shared" si="23"/>
+        <v>1.5714285714285714</v>
+      </c>
+      <c r="O56">
+        <f t="shared" si="24"/>
+        <v>39.5</v>
+      </c>
+      <c r="P56">
+        <f t="shared" si="25"/>
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="Q56">
+        <f t="shared" si="26"/>
+        <v>0</v>
+      </c>
+      <c r="S56">
+        <f t="shared" si="27"/>
+        <v>0.24</v>
+      </c>
+      <c r="T56">
+        <f t="shared" si="28"/>
+        <v>0.11</v>
+      </c>
+      <c r="U56">
+        <f t="shared" si="29"/>
+        <v>0.6784</v>
+      </c>
+      <c r="W56">
+        <f t="shared" si="18"/>
+        <v>0.79</v>
+      </c>
+      <c r="X56">
+        <f t="shared" si="30"/>
+        <v>0</v>
+      </c>
+      <c r="Y56">
+        <f t="shared" si="31"/>
+        <v>4.7000000000000002E-3</v>
+      </c>
+      <c r="Z56">
+        <f t="shared" si="32"/>
+        <v>1.6538645760000002E-3</v>
+      </c>
+      <c r="AA56">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="AB56">
+        <f t="shared" si="34"/>
+        <v>12.0732114048</v>
+      </c>
+      <c r="AC56">
+        <f t="shared" si="35"/>
+        <v>1.2073211404800001E-2</v>
+      </c>
+    </row>
+    <row r="57" spans="1:34">
+      <c r="A57" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C57">
+        <v>21</v>
+      </c>
+      <c r="D57" t="s">
+        <v>56</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F57">
+        <v>26</v>
+      </c>
+      <c r="H57" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="I57">
+        <f t="shared" si="19"/>
+        <v>0.34</v>
+      </c>
+      <c r="J57">
+        <f t="shared" si="20"/>
+        <v>0.19</v>
+      </c>
+      <c r="K57" t="s">
+        <v>56</v>
+      </c>
+      <c r="L57">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="M57">
+        <f t="shared" si="22"/>
+        <v>1</v>
+      </c>
+      <c r="N57">
+        <f t="shared" si="23"/>
+        <v>1.5714285714285714</v>
+      </c>
+      <c r="O57">
+        <f t="shared" si="24"/>
+        <v>7</v>
+      </c>
+      <c r="P57">
+        <f t="shared" si="25"/>
+        <v>1.9900000000000001E-2</v>
+      </c>
+      <c r="Q57">
+        <f t="shared" si="26"/>
+        <v>1</v>
+      </c>
+      <c r="S57">
+        <f t="shared" si="27"/>
+        <v>0.24</v>
+      </c>
+      <c r="T57">
+        <f t="shared" si="28"/>
+        <v>0.11</v>
+      </c>
+      <c r="U57">
+        <f t="shared" si="29"/>
+        <v>0.6784</v>
+      </c>
+      <c r="W57">
+        <f t="shared" si="18"/>
+        <v>0.79</v>
+      </c>
+      <c r="X57">
+        <f t="shared" si="30"/>
+        <v>0</v>
+      </c>
+      <c r="Y57">
+        <f t="shared" si="31"/>
+        <v>4.7000000000000002E-3</v>
+      </c>
+      <c r="Z57">
+        <f t="shared" si="32"/>
+        <v>2.0597580800000003E-4</v>
+      </c>
+      <c r="AA57">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="AB57">
+        <f t="shared" si="34"/>
+        <v>1.57880456832</v>
+      </c>
+      <c r="AC57">
+        <f t="shared" si="35"/>
+        <v>1.5788045683200001E-3</v>
+      </c>
+    </row>
+    <row r="58" spans="1:34">
+      <c r="A58" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C58">
+        <v>22</v>
+      </c>
+      <c r="D58" t="s">
+        <v>57</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F58">
+        <v>27</v>
+      </c>
+      <c r="H58" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="I58">
+        <f t="shared" si="19"/>
+        <v>2.73</v>
+      </c>
+      <c r="J58">
+        <f t="shared" si="20"/>
+        <v>0.19</v>
+      </c>
+      <c r="K58" t="s">
+        <v>56</v>
+      </c>
+      <c r="L58">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="M58">
+        <f t="shared" si="22"/>
+        <v>1</v>
+      </c>
+      <c r="N58">
+        <f t="shared" si="23"/>
+        <v>1.5714285714285714</v>
+      </c>
+      <c r="O58">
+        <f t="shared" si="24"/>
+        <v>39.5</v>
+      </c>
+      <c r="P58">
+        <f t="shared" si="25"/>
+        <v>5.3E-3</v>
+      </c>
+      <c r="Q58">
+        <f t="shared" si="26"/>
+        <v>0</v>
+      </c>
+      <c r="S58">
+        <f t="shared" si="27"/>
+        <v>0.24</v>
+      </c>
+      <c r="T58">
+        <f t="shared" si="28"/>
+        <v>0.11</v>
+      </c>
+      <c r="U58">
+        <f t="shared" si="29"/>
+        <v>0.6784</v>
+      </c>
+      <c r="W58">
+        <f t="shared" si="18"/>
+        <v>0.8</v>
+      </c>
+      <c r="X58">
+        <f t="shared" si="30"/>
+        <v>0</v>
+      </c>
+      <c r="Y58">
+        <f t="shared" si="31"/>
+        <v>4.7000000000000002E-3</v>
+      </c>
+      <c r="Z58">
+        <f t="shared" si="32"/>
+        <v>1.6538645760000002E-3</v>
+      </c>
+      <c r="AA58">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="AB58">
+        <f t="shared" si="34"/>
+        <v>13.28053254528</v>
+      </c>
+      <c r="AC58">
+        <f t="shared" si="35"/>
+        <v>1.3280532545279999E-2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:34">
+      <c r="A59" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C59">
+        <v>23</v>
+      </c>
+      <c r="D59" t="s">
+        <v>56</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="F59" t="s">
+        <v>92</v>
+      </c>
+      <c r="H59" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="I59">
+        <f t="shared" si="19"/>
+        <v>0.91</v>
+      </c>
+      <c r="J59">
+        <f t="shared" si="20"/>
+        <v>0.19</v>
+      </c>
+      <c r="K59" t="s">
+        <v>56</v>
+      </c>
+      <c r="L59">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="M59">
+        <f t="shared" si="22"/>
+        <v>1</v>
+      </c>
+      <c r="N59">
+        <f t="shared" si="23"/>
+        <v>1.5714285714285714</v>
+      </c>
+      <c r="O59">
+        <f t="shared" si="24"/>
+        <v>13.2</v>
+      </c>
+      <c r="P59">
+        <f t="shared" si="25"/>
+        <v>6.4000000000000003E-3</v>
+      </c>
+      <c r="Q59">
+        <f t="shared" si="26"/>
+        <v>1</v>
+      </c>
+      <c r="S59">
+        <f t="shared" si="27"/>
+        <v>0.24</v>
+      </c>
+      <c r="T59">
+        <f t="shared" si="28"/>
+        <v>0.11</v>
+      </c>
+      <c r="U59">
+        <f t="shared" si="29"/>
+        <v>0.6784</v>
+      </c>
+      <c r="W59">
+        <f t="shared" si="18"/>
+        <v>0.8</v>
+      </c>
+      <c r="X59">
+        <f t="shared" si="30"/>
+        <v>0</v>
+      </c>
+      <c r="Y59">
+        <f t="shared" si="31"/>
+        <v>4.7000000000000002E-3</v>
+      </c>
+      <c r="Z59">
+        <f t="shared" si="32"/>
+        <v>5.5128819200000003E-4</v>
+      </c>
+      <c r="AA59">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="AB59">
+        <f t="shared" si="34"/>
+        <v>4.6280643718399999</v>
+      </c>
+      <c r="AC59">
+        <f t="shared" si="35"/>
+        <v>4.6280643718400001E-3</v>
+      </c>
+    </row>
+    <row r="60" spans="1:34">
+      <c r="A60" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C60">
+        <v>24</v>
+      </c>
+      <c r="D60" t="s">
+        <v>57</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="F60">
+        <v>20</v>
+      </c>
+      <c r="H60" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="I60">
+        <f t="shared" si="19"/>
+        <v>0.34</v>
+      </c>
+      <c r="J60">
+        <f t="shared" si="20"/>
+        <v>0.19</v>
+      </c>
+      <c r="K60" t="s">
+        <v>56</v>
+      </c>
+      <c r="L60">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="M60">
+        <f t="shared" si="22"/>
+        <v>1</v>
+      </c>
+      <c r="N60">
+        <f t="shared" si="23"/>
+        <v>1.5714285714285714</v>
+      </c>
+      <c r="O60">
+        <f t="shared" si="24"/>
+        <v>7</v>
+      </c>
+      <c r="P60">
+        <f t="shared" si="25"/>
+        <v>2.5999999999999999E-3</v>
+      </c>
+      <c r="Q60">
+        <f t="shared" si="26"/>
+        <v>0</v>
+      </c>
+      <c r="S60">
+        <f t="shared" si="27"/>
+        <v>0.24</v>
+      </c>
+      <c r="T60">
+        <f t="shared" si="28"/>
+        <v>0.11</v>
+      </c>
+      <c r="U60">
+        <f t="shared" si="29"/>
+        <v>0.6784</v>
+      </c>
+      <c r="W60">
+        <f t="shared" si="18"/>
+        <v>0.78</v>
+      </c>
+      <c r="X60">
+        <f t="shared" si="30"/>
+        <v>0</v>
+      </c>
+      <c r="Y60">
+        <f t="shared" si="31"/>
+        <v>4.7000000000000002E-3</v>
+      </c>
+      <c r="Z60">
+        <f t="shared" si="32"/>
+        <v>2.0597580800000003E-4</v>
+      </c>
+      <c r="AA60">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="AB60">
+        <f t="shared" si="34"/>
+        <v>1.8043480780800005</v>
+      </c>
+      <c r="AC60">
+        <f t="shared" si="35"/>
+        <v>1.8043480780800005E-3</v>
+      </c>
+    </row>
+    <row r="61" spans="1:34">
+      <c r="E61" s="2"/>
+    </row>
+    <row r="62" spans="1:34">
+      <c r="E62" s="2"/>
+    </row>
+    <row r="63" spans="1:34">
+      <c r="E63" s="2"/>
+    </row>
+    <row r="64" spans="1:34">
+      <c r="E64" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>